<commit_message>
feat: add Zoho Books integration, CRM endpoints, sample data seeders, and documentation
</commit_message>
<xml_diff>
--- a/sample_rfq_bom_costing.xlsx
+++ b/sample_rfq_bom_costing.xlsx
@@ -6,6 +6,10 @@
     <sheet name="RFQ" sheetId="1" r:id="rId1"/>
     <sheet name="BOM" sheetId="2" r:id="rId2"/>
     <sheet name="Costing" sheetId="3" r:id="rId3"/>
+    <sheet name="Quotes" sheetId="4" r:id="rId4"/>
+    <sheet name="Sales Orders" sheetId="5" r:id="rId5"/>
+    <sheet name="Invoices" sheetId="6" r:id="rId6"/>
+    <sheet name="Vendors" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -845,4 +849,875 @@
     <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:Q4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Quote Number</v>
+      </c>
+      <c r="B1" t="str">
+        <v>RFQ Number</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Customer ID</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Customer Name</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Contact Person</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Email</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Phone</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Issue Date</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Expiry Date</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Subtotal</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Tax Rate Pct</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Tax Amount</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Total Amount</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Payment Terms</v>
+      </c>
+      <c r="P1" t="str">
+        <v>Validity Days</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>QUO-2026-001</v>
+      </c>
+      <c r="B2" t="str">
+        <v>RFQ-2026-003</v>
+      </c>
+      <c r="C2" t="str">
+        <v>c-3</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Crestline Switchgear</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Vikram Shah</v>
+      </c>
+      <c r="F2" t="str">
+        <v>vikram@crestlineswitchgear.com</v>
+      </c>
+      <c r="G2" t="str">
+        <v>+91 98901 55567</v>
+      </c>
+      <c r="H2" t="str">
+        <v>2026-10-23</v>
+      </c>
+      <c r="I2" t="str">
+        <v>2026-11-23</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Sent</v>
+      </c>
+      <c r="K2">
+        <v>97980</v>
+      </c>
+      <c r="L2">
+        <v>18</v>
+      </c>
+      <c r="M2">
+        <v>17636.4</v>
+      </c>
+      <c r="N2">
+        <v>115616.4</v>
+      </c>
+      <c r="O2" t="str">
+        <v>50% advance, balance against PI before dispatch</v>
+      </c>
+      <c r="P2">
+        <v>30</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Includes 1-year on-site replacement warranty. Lead time 3 weeks.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>QUO-2026-002</v>
+      </c>
+      <c r="B3" t="str">
+        <v>RFQ-2026-002</v>
+      </c>
+      <c r="C3" t="str">
+        <v>c-2</v>
+      </c>
+      <c r="D3" t="str">
+        <v>BluePeak Automation</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Neha Verma</v>
+      </c>
+      <c r="F3" t="str">
+        <v>neha@bluepeakautomation.in</v>
+      </c>
+      <c r="G3" t="str">
+        <v>+91 98200 11223</v>
+      </c>
+      <c r="H3" t="str">
+        <v>2026-10-20</v>
+      </c>
+      <c r="I3" t="str">
+        <v>2026-11-20</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Converted to Order</v>
+      </c>
+      <c r="K3">
+        <v>124000</v>
+      </c>
+      <c r="L3">
+        <v>18</v>
+      </c>
+      <c r="M3">
+        <v>22320</v>
+      </c>
+      <c r="N3">
+        <v>146320</v>
+      </c>
+      <c r="O3" t="str">
+        <v>Net 30 days</v>
+      </c>
+      <c r="P3">
+        <v>30</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>Customer approved quote. Released under Sales Order SO-2026-015.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>QUO-2026-003</v>
+      </c>
+      <c r="B4" t="str">
+        <v>RFQ-2026-083</v>
+      </c>
+      <c r="C4" t="str">
+        <v>c-0083</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Delta Automation Tech</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Siddharth Rao</v>
+      </c>
+      <c r="F4" t="str">
+        <v>siddharth@deltaautomation.in</v>
+      </c>
+      <c r="G4" t="str">
+        <v>+91 98450 12345</v>
+      </c>
+      <c r="H4" t="str">
+        <v>2026-10-26</v>
+      </c>
+      <c r="I4" t="str">
+        <v>2026-11-15</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Approved</v>
+      </c>
+      <c r="K4">
+        <v>360000</v>
+      </c>
+      <c r="L4">
+        <v>18</v>
+      </c>
+      <c r="M4">
+        <v>64800</v>
+      </c>
+      <c r="N4">
+        <v>424800</v>
+      </c>
+      <c r="O4" t="str">
+        <v>30% advance, 70% Net 30</v>
+      </c>
+      <c r="P4">
+        <v>20</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>Technical clearance approved. Dispatched for PO issuance.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:O4"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Sales Order Number</v>
+      </c>
+      <c r="B1" t="str">
+        <v>RFQ Number</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Customer ID</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Customer Name</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Order Date</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Shipment Date</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Status</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Subtotal</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Tax Amount</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Shipping Charges</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Total Amount</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Billing City</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Billing State</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Notes</v>
+      </c>
+      <c r="O1" t="str">
+        <v>Quote Number</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>SO-2026-014</v>
+      </c>
+      <c r="B2" t="str">
+        <v>RFQ-2026-006</v>
+      </c>
+      <c r="C2" t="str">
+        <v>c-6</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Fabricate One</v>
+      </c>
+      <c r="E2" t="str">
+        <v>2026-10-21</v>
+      </c>
+      <c r="F2" t="str">
+        <v>2026-11-22</v>
+      </c>
+      <c r="G2" t="str">
+        <v>In Production</v>
+      </c>
+      <c r="H2">
+        <v>186500</v>
+      </c>
+      <c r="I2">
+        <v>33570</v>
+      </c>
+      <c r="J2">
+        <v>2500</v>
+      </c>
+      <c r="K2">
+        <v>222570</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Bengaluru</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Karnataka</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Scheduled in Bay 3. Billed under INV-2026-091.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>SO-2026-015</v>
+      </c>
+      <c r="B3" t="str">
+        <v>RFQ-2026-002</v>
+      </c>
+      <c r="C3" t="str">
+        <v>c-2</v>
+      </c>
+      <c r="D3" t="str">
+        <v>BluePeak Automation</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2026-10-26</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2026-11-12</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Confirmed</v>
+      </c>
+      <c r="H3">
+        <v>124000</v>
+      </c>
+      <c r="I3">
+        <v>22320</v>
+      </c>
+      <c r="J3">
+        <v>1800</v>
+      </c>
+      <c r="K3">
+        <v>148120</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Pune</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Maharashtra</v>
+      </c>
+      <c r="N3" t="str">
+        <v>PO received. Invoiced under INV-2026-092.</v>
+      </c>
+      <c r="O3" t="str">
+        <v>QUO-2026-002</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>SO-2026-016</v>
+      </c>
+      <c r="B4" t="str">
+        <v>RFQ-2026-083</v>
+      </c>
+      <c r="C4" t="str">
+        <v>c-0083</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Delta Automation Tech</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2026-10-28</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2026-11-20</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Confirmed</v>
+      </c>
+      <c r="H4">
+        <v>360000</v>
+      </c>
+      <c r="I4">
+        <v>64800</v>
+      </c>
+      <c r="J4">
+        <v>4000</v>
+      </c>
+      <c r="K4">
+        <v>428800</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Chennai</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Tamil Nadu</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Signed purchase confirmation received.</v>
+      </c>
+      <c r="O4" t="str">
+        <v>QUO-2026-003</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:O4"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:N5"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Invoice Number</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Sales Order Number</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Customer ID</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Customer Name</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Invoice Date</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Due Date</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Payment Status</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Payment Terms</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Subtotal</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Tax Amount</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Total Amount</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Paid Amount</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Balance Due</v>
+      </c>
+      <c r="N1" t="str">
+        <v>Notes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>INV-2026-091</v>
+      </c>
+      <c r="B2" t="str">
+        <v>SO-2026-014</v>
+      </c>
+      <c r="C2" t="str">
+        <v>c-6</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Fabricate One</v>
+      </c>
+      <c r="E2" t="str">
+        <v>2026-10-22</v>
+      </c>
+      <c r="F2" t="str">
+        <v>2026-11-21</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Partially Paid</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Net 30</v>
+      </c>
+      <c r="I2">
+        <v>186500</v>
+      </c>
+      <c r="J2">
+        <v>33570</v>
+      </c>
+      <c r="K2">
+        <v>220070</v>
+      </c>
+      <c r="L2">
+        <v>110000</v>
+      </c>
+      <c r="M2">
+        <v>110070</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Advance payment of INR 1,10,000 received via NEFT/RTGS.</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>INV-2026-092</v>
+      </c>
+      <c r="B3" t="str">
+        <v>SO-2026-015</v>
+      </c>
+      <c r="C3" t="str">
+        <v>c-2</v>
+      </c>
+      <c r="D3" t="str">
+        <v>BluePeak Automation</v>
+      </c>
+      <c r="E3" t="str">
+        <v>2026-10-27</v>
+      </c>
+      <c r="F3" t="str">
+        <v>2026-11-26</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Unpaid</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Net 30</v>
+      </c>
+      <c r="I3">
+        <v>124000</v>
+      </c>
+      <c r="J3">
+        <v>22320</v>
+      </c>
+      <c r="K3">
+        <v>146320</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>146320</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Tax invoice sent to finance team for processing.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>INV-2026-090</v>
+      </c>
+      <c r="B4" t="str">
+        <v>SO-2026-017</v>
+      </c>
+      <c r="C4" t="str">
+        <v>c-1</v>
+      </c>
+      <c r="D4" t="str">
+        <v>Aarav Controls</v>
+      </c>
+      <c r="E4" t="str">
+        <v>2026-10-15</v>
+      </c>
+      <c r="F4" t="str">
+        <v>2026-10-30</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Paid</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Net 15</v>
+      </c>
+      <c r="I4">
+        <v>85500</v>
+      </c>
+      <c r="J4">
+        <v>15390</v>
+      </c>
+      <c r="K4">
+        <v>100890</v>
+      </c>
+      <c r="L4">
+        <v>100890</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Full payment received on 2026-10-28 via IMPS ref #9081234.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>INV-2026-093</v>
+      </c>
+      <c r="B5" t="str">
+        <v>SO-2026-016</v>
+      </c>
+      <c r="C5" t="str">
+        <v>c-0083</v>
+      </c>
+      <c r="D5" t="str">
+        <v>Delta Automation Tech</v>
+      </c>
+      <c r="E5" t="str">
+        <v>2026-10-28</v>
+      </c>
+      <c r="F5" t="str">
+        <v>2026-11-27</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Partially Paid</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Net 30</v>
+      </c>
+      <c r="I5">
+        <v>360000</v>
+      </c>
+      <c r="J5">
+        <v>64800</v>
+      </c>
+      <c r="K5">
+        <v>424800</v>
+      </c>
+      <c r="L5">
+        <v>127440</v>
+      </c>
+      <c r="M5">
+        <v>297360</v>
+      </c>
+      <c r="N5" t="str">
+        <v>30% advance milestone paid.</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:N5"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:K6"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Vendor ID</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Vendor Name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Contact Person</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Email</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Phone</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Category</v>
+      </c>
+      <c r="G1" t="str">
+        <v>GSTIN</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Payment Terms</v>
+      </c>
+      <c r="I1" t="str">
+        <v>City</v>
+      </c>
+      <c r="J1" t="str">
+        <v>State</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Status</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>v-101</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Precision Steel &amp; Alloys Ltd</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Amit Verma</v>
+      </c>
+      <c r="D2" t="str">
+        <v>amit@precisionsteel.in</v>
+      </c>
+      <c r="E2" t="str">
+        <v>+91 98200 44556</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Raw Materials &amp; Metals</v>
+      </c>
+      <c r="G2" t="str">
+        <v>27AABCP1234F1Z5</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Net 30</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Pune</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Maharashtra</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>v-102</v>
+      </c>
+      <c r="B3" t="str">
+        <v>TechnoCore CNC Machining Works</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Rakesh Sharma</v>
+      </c>
+      <c r="D3" t="str">
+        <v>rakesh@technocore-cnc.com</v>
+      </c>
+      <c r="E3" t="str">
+        <v>+91 97110 88231</v>
+      </c>
+      <c r="F3" t="str">
+        <v>CNC Machining &amp; Tooling</v>
+      </c>
+      <c r="G3" t="str">
+        <v>29AABCT5678M1Z2</v>
+      </c>
+      <c r="H3" t="str">
+        <v>Net 45</v>
+      </c>
+      <c r="I3" t="str">
+        <v>Bengaluru</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Karnataka</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>v-103</v>
+      </c>
+      <c r="B4" t="str">
+        <v>ElectraMotion Dynamics Pvt Ltd</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Meera Krishnan</v>
+      </c>
+      <c r="D4" t="str">
+        <v>meera@electramotion.co</v>
+      </c>
+      <c r="E4" t="str">
+        <v>+91 98450 77112</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Motors &amp; Actuators</v>
+      </c>
+      <c r="G4" t="str">
+        <v>33AABCE9012K1Z8</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Net 15</v>
+      </c>
+      <c r="I4" t="str">
+        <v>Chennai</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Tamil Nadu</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>v-104</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Zenith Fasteners &amp; Hardware</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Dilip Patel</v>
+      </c>
+      <c r="D5" t="str">
+        <v>dilip@zenithfasteners.in</v>
+      </c>
+      <c r="E5" t="str">
+        <v>+91 98980 33211</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Industrial Hardware &amp; Fasteners</v>
+      </c>
+      <c r="G5" t="str">
+        <v>24AABCZ3456L1Z4</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Advance</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Ahmedabad</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Gujarat</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>v-105</v>
+      </c>
+      <c r="B6" t="str">
+        <v>OptiSensor Technologies</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Sneha Roy</v>
+      </c>
+      <c r="D6" t="str">
+        <v>sneha@optisensor.io</v>
+      </c>
+      <c r="E6" t="str">
+        <v>+91 98310 99443</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Sensors &amp; Instrumentation</v>
+      </c>
+      <c r="G6" t="str">
+        <v>19AABCO7890N1Z9</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Net 30</v>
+      </c>
+      <c r="I6" t="str">
+        <v>Kolkata</v>
+      </c>
+      <c r="J6" t="str">
+        <v>West Bengal</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Active</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:K6"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>